<commit_message>
MAJ modèles logiques : FRLMProblem et FRLMDevice 8612777a96f8e46a73b4e0100d7f533884dd5f29
</commit_message>
<xml_diff>
--- a/modeleLogiqueSBM/ig/StructureDefinition-fr-lm-antecedents-medicaux.xlsx
+++ b/modeleLogiqueSBM/ig/StructureDefinition-fr-lm-antecedents-medicaux.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-07T14:19:51+00:00</t>
+    <t>2026-04-07T14:45:49+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -317,7 +317,7 @@
     <t>fr-lm-antecedents-medicaux.entree.problemes</t>
   </si>
   <si>
-    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-problem
+    <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-lm-condition
 </t>
   </si>
   <si>
@@ -636,7 +636,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="65.3125" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="66.0390625" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>

</xml_diff>